<commit_message>
performance optimization; excel upload for online eegs
</commit_message>
<xml_diff>
--- a/tests/TE100200-Muster-Stammdatenimport.xlsx
+++ b/tests/TE100200-Muster-Stammdatenimport.xlsx
@@ -150,7 +150,7 @@
     <t xml:space="preserve">37</t>
   </si>
   <si>
-    <t xml:space="preserve">AT00999900000000000000000000101</t>
+    <t xml:space="preserve">AT0099990000000000000000000000101</t>
   </si>
   <si>
     <t xml:space="preserve">CONSUMPTION</t>
@@ -186,7 +186,7 @@
     <t xml:space="preserve">Baumallee</t>
   </si>
   <si>
-    <t xml:space="preserve">AT00000000000000000000000000001</t>
+    <t xml:space="preserve">AT0000000000000000000000000000001</t>
   </si>
   <si>
     <t xml:space="preserve">GENERATION</t>
@@ -210,7 +210,7 @@
     <t xml:space="preserve">35</t>
   </si>
   <si>
-    <t xml:space="preserve">AT00000000000000000000000000002</t>
+    <t xml:space="preserve">AT0000000000000000000000000000002</t>
   </si>
   <si>
     <t xml:space="preserve">ZP003</t>
@@ -231,7 +231,7 @@
     <t xml:space="preserve">003</t>
   </si>
   <si>
-    <t xml:space="preserve">AT00000000000000000000000000003</t>
+    <t xml:space="preserve">AT0000000000000000000000000000003</t>
   </si>
   <si>
     <t xml:space="preserve">ZP004</t>
@@ -249,7 +249,7 @@
     <t xml:space="preserve">70</t>
   </si>
   <si>
-    <t xml:space="preserve">AT00000000000000000000000000004</t>
+    <t xml:space="preserve">AT0000000000000000000000000000004</t>
   </si>
   <si>
     <t xml:space="preserve">ZP005</t>
@@ -270,7 +270,7 @@
     <t xml:space="preserve">22</t>
   </si>
   <si>
-    <t xml:space="preserve">AT00000000000000000000000000005</t>
+    <t xml:space="preserve">AT0000000000000000000000000000005</t>
   </si>
   <si>
     <t xml:space="preserve">ZP006</t>
@@ -288,7 +288,7 @@
     <t xml:space="preserve">Picknickstraße</t>
   </si>
   <si>
-    <t xml:space="preserve">AT00000000000000000000000000006</t>
+    <t xml:space="preserve">AT0000000000000000000000000000006</t>
   </si>
   <si>
     <t xml:space="preserve">ZP007</t>
@@ -303,7 +303,7 @@
     <t xml:space="preserve">24</t>
   </si>
   <si>
-    <t xml:space="preserve">AT00000000000000000000000000007</t>
+    <t xml:space="preserve">AT0000000000000000000000000000007</t>
   </si>
   <si>
     <t xml:space="preserve">ZP008</t>
@@ -324,7 +324,7 @@
     <t xml:space="preserve">NEW</t>
   </si>
   <si>
-    <t xml:space="preserve">AT00000000000000000000000000008</t>
+    <t xml:space="preserve">AT0000000000000000000000000000008</t>
   </si>
   <si>
     <t xml:space="preserve">ZP009</t>
@@ -339,7 +339,7 @@
     <t xml:space="preserve">23</t>
   </si>
   <si>
-    <t xml:space="preserve">AT00000000000000000000000000009</t>
+    <t xml:space="preserve">AT0000000000000000000000000000009</t>
   </si>
   <si>
     <t xml:space="preserve">ZP010</t>
@@ -354,7 +354,7 @@
     <t xml:space="preserve">010</t>
   </si>
   <si>
-    <t xml:space="preserve">AT00000000000000000000000000010</t>
+    <t xml:space="preserve">AT0000000000000000000000000000010</t>
   </si>
   <si>
     <t xml:space="preserve">ZP011</t>
@@ -517,7 +517,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AA20"/>
-  <sheetFormatPr defaultColWidth="10.8125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.82421875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="37.16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34.47"/>
@@ -1408,7 +1408,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:M1"/>
-  <sheetFormatPr defaultColWidth="10.8125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.82421875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5.2"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="5.04"/>

</xml_diff>